<commit_message>
Clustering: general clusters = one page; clarify column semantics
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016UEhV6w824sjkUhMCvDZb2
</commit_message>
<xml_diff>
--- a/clustering_t-ind.ru.xlsx
+++ b/clustering_t-ind.ru.xlsx
@@ -496,12 +496,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Хаб-категория: «оборудование для шиномонтажа купить/цена/магазин/аппарат» — единая SERP-группа (avto-master, mactak, vilse); одна коммерческая страница. (запросов в кластере: 12, сумма частотности: 1889)</t>
+          <t>Все запросы — варианты одного коммерческого запроса («оборудование», «купить», «цена», «магазин», «в Москве/СПб»), в SERP единая группа (avto-master, mactak, vilse): ведём на одну страницу — главную категорию оборудования. (запросов в кластере: 12, сумма частотности: 1889)</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -531,12 +531,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Хаб-категория: «оборудование для шиномонтажа купить/цена/магазин/аппарат» — единая SERP-группа (avto-master, mactak, vilse); одна коммерческая страница. (запросов в кластере: 12, сумма частотности: 1889)</t>
+          <t>Все запросы — варианты одного коммерческого запроса («оборудование», «купить», «цена», «магазин», «в Москве/СПб»), в SERP единая группа (avto-master, mactak, vilse): ведём на одну страницу — главную категорию оборудования. (запросов в кластере: 12, сумма частотности: 1889)</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -566,12 +566,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Хаб-категория: «оборудование для шиномонтажа купить/цена/магазин/аппарат» — единая SERP-группа (avto-master, mactak, vilse); одна коммерческая страница. (запросов в кластере: 12, сумма частотности: 1889)</t>
+          <t>Все запросы — варианты одного коммерческого запроса («оборудование», «купить», «цена», «магазин», «в Москве/СПб»), в SERP единая группа (avto-master, mactak, vilse): ведём на одну страницу — главную категорию оборудования. (запросов в кластере: 12, сумма частотности: 1889)</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -601,12 +601,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Хаб-категория: «оборудование для шиномонтажа купить/цена/магазин/аппарат» — единая SERP-группа (avto-master, mactak, vilse); одна коммерческая страница. (запросов в кластере: 12, сумма частотности: 1889)</t>
+          <t>Все запросы — варианты одного коммерческого запроса («оборудование», «купить», «цена», «магазин», «в Москве/СПб»), в SERP единая группа (avto-master, mactak, vilse): ведём на одну страницу — главную категорию оборудования. (запросов в кластере: 12, сумма частотности: 1889)</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -636,12 +636,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Хаб-категория: «оборудование для шиномонтажа купить/цена/магазин/аппарат» — единая SERP-группа (avto-master, mactak, vilse); одна коммерческая страница. (запросов в кластере: 12, сумма частотности: 1889)</t>
+          <t>Все запросы — варианты одного коммерческого запроса («оборудование», «купить», «цена», «магазин», «в Москве/СПб»), в SERP единая группа (avto-master, mactak, vilse): ведём на одну страницу — главную категорию оборудования. (запросов в кластере: 12, сумма частотности: 1889)</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -671,12 +671,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Хаб-категория: «оборудование для шиномонтажа купить/цена/магазин/аппарат» — единая SERP-группа (avto-master, mactak, vilse); одна коммерческая страница. (запросов в кластере: 12, сумма частотности: 1889)</t>
+          <t>Все запросы — варианты одного коммерческого запроса («оборудование», «купить», «цена», «магазин», «в Москве/СПб»), в SERP единая группа (avto-master, mactak, vilse): ведём на одну страницу — главную категорию оборудования. (запросов в кластере: 12, сумма частотности: 1889)</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -706,12 +706,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Хаб-категория: «оборудование для шиномонтажа купить/цена/магазин/аппарат» — единая SERP-группа (avto-master, mactak, vilse); одна коммерческая страница. (запросов в кластере: 12, сумма частотности: 1889)</t>
+          <t>Все запросы — варианты одного коммерческого запроса («оборудование», «купить», «цена», «магазин», «в Москве/СПб»), в SERP единая группа (avto-master, mactak, vilse): ведём на одну страницу — главную категорию оборудования. (запросов в кластере: 12, сумма частотности: 1889)</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -741,12 +741,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Хаб-категория: «оборудование для шиномонтажа купить/цена/магазин/аппарат» — единая SERP-группа (avto-master, mactak, vilse); одна коммерческая страница. (запросов в кластере: 12, сумма частотности: 1889)</t>
+          <t>Все запросы — варианты одного коммерческого запроса («оборудование», «купить», «цена», «магазин», «в Москве/СПб»), в SERP единая группа (avto-master, mactak, vilse): ведём на одну страницу — главную категорию оборудования. (запросов в кластере: 12, сумма частотности: 1889)</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -776,12 +776,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Хаб-категория: «оборудование для шиномонтажа купить/цена/магазин/аппарат» — единая SERP-группа (avto-master, mactak, vilse); одна коммерческая страница. (запросов в кластере: 12, сумма частотности: 1889)</t>
+          <t>Все запросы — варианты одного коммерческого запроса («оборудование», «купить», «цена», «магазин», «в Москве/СПб»), в SERP единая группа (avto-master, mactak, vilse): ведём на одну страницу — главную категорию оборудования. (запросов в кластере: 12, сумма частотности: 1889)</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -916,12 +916,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Основная коммерческая страница по станкам: «станок/стенд купить», «станок для шиномонтажа», «в Москве» — один набор URL в SERP (vsedlyasto, technovector, vilse) — объединяем в одну страницу. (запросов в кластере: 6, сумма частотности: 1564)</t>
+          <t>Все запросы — варианты одного коммерческого запроса («станок/стенд», «купить», «в Москве»), в SERP один набор URL (vsedlyasto, technovector, vilse): ведём на одну страницу со станками. (запросов в кластере: 6, сумма частотности: 1564)</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -951,12 +951,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Основная коммерческая страница по станкам: «станок/стенд купить», «станок для шиномонтажа», «в Москве» — один набор URL в SERP (vsedlyasto, technovector, vilse) — объединяем в одну страницу. (запросов в кластере: 6, сумма частотности: 1564)</t>
+          <t>Все запросы — варианты одного коммерческого запроса («станок/стенд», «купить», «в Москве»), в SERP один набор URL (vsedlyasto, technovector, vilse): ведём на одну страницу со станками. (запросов в кластере: 6, сумма частотности: 1564)</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -986,12 +986,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Основная коммерческая страница по станкам: «станок/стенд купить», «станок для шиномонтажа», «в Москве» — один набор URL в SERP (vsedlyasto, technovector, vilse) — объединяем в одну страницу. (запросов в кластере: 6, сумма частотности: 1564)</t>
+          <t>Все запросы — варианты одного коммерческого запроса («станок/стенд», «купить», «в Москве»), в SERP один набор URL (vsedlyasto, technovector, vilse): ведём на одну страницу со станками. (запросов в кластере: 6, сумма частотности: 1564)</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -1021,12 +1021,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Основная коммерческая страница по станкам: «станок/стенд купить», «станок для шиномонтажа», «в Москве» — один набор URL в SERP (vsedlyasto, technovector, vilse) — объединяем в одну страницу. (запросов в кластере: 6, сумма частотности: 1564)</t>
+          <t>Все запросы — варианты одного коммерческого запроса («станок/стенд», «купить», «в Москве»), в SERP один набор URL (vsedlyasto, technovector, vilse): ведём на одну страницу со станками. (запросов в кластере: 6, сумма частотности: 1564)</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -1056,12 +1056,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Основная коммерческая страница по станкам: «станок/стенд купить», «станок для шиномонтажа», «в Москве» — один набор URL в SERP (vsedlyasto, technovector, vilse) — объединяем в одну страницу. (запросов в кластере: 6, сумма частотности: 1564)</t>
+          <t>Все запросы — варианты одного коммерческого запроса («станок/стенд», «купить», «в Москве»), в SERP один набор URL (vsedlyasto, technovector, vilse): ведём на одну страницу со станками. (запросов в кластере: 6, сумма частотности: 1564)</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -1091,12 +1091,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Основная коммерческая страница по станкам: «станок/стенд купить», «станок для шиномонтажа», «в Москве» — один набор URL в SERP (vsedlyasto, technovector, vilse) — объединяем в одну страницу. (запросов в кластере: 6, сумма частотности: 1564)</t>
+          <t>Все запросы — варианты одного коммерческого запроса («станок/стенд», «купить», «в Москве»), в SERP один набор URL (vsedlyasto, technovector, vilse): ведём на одну страницу со станками. (запросов в кластере: 6, сумма частотности: 1564)</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -4171,12 +4171,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E107" t="n">
@@ -4206,12 +4206,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E108" t="n">
@@ -4241,12 +4241,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E109" t="n">
@@ -4276,12 +4276,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E110" t="n">
@@ -4311,12 +4311,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E111" t="n">
@@ -4346,12 +4346,12 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E112" t="n">
@@ -4381,12 +4381,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E113" t="n">
@@ -4416,12 +4416,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E114" t="n">
@@ -4451,12 +4451,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E115" t="n">
@@ -4486,12 +4486,12 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E116" t="n">
@@ -4521,12 +4521,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E117" t="n">
@@ -4556,12 +4556,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E118" t="n">
@@ -4591,12 +4591,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E119" t="n">
@@ -4626,12 +4626,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E120" t="n">
@@ -4661,12 +4661,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E121" t="n">
@@ -4696,12 +4696,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E122" t="n">
@@ -4731,12 +4731,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E123" t="n">
@@ -4766,12 +4766,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E124" t="n">
@@ -4801,12 +4801,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E125" t="n">
@@ -4836,12 +4836,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -4871,12 +4871,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -4906,12 +4906,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -4941,12 +4941,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E129" t="n">
@@ -4976,12 +4976,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E130" t="n">
@@ -5011,12 +5011,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Отдельная посадочная</t>
+          <t>Одна страница</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>Крупнейшая SERP-группа (21 запрос): станок/стенд/оборудование/аппарат для балансировки, «купить», «цена», для легковых — один набор URL; объединяем на одной коммерческой странице каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
+          <t>Все запросы — синонимы и коммерческие варианты («станок/стенд/аппарат», «купить», «цена», для легковых): крупнейшая группа выдачи (21 запрос) с одним набором URL — ведём на одну страницу каталога. (запросов в кластере: 25, сумма частотности: 1290)</t>
         </is>
       </c>
       <c r="E131" t="n">
@@ -7578,7 +7578,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -7611,7 +7611,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -7677,7 +7677,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -7710,7 +7710,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -7743,7 +7743,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -7776,7 +7776,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -7809,7 +7809,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -7842,7 +7842,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -7875,7 +7875,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -7908,7 +7908,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -7941,7 +7941,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -7974,7 +7974,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8007,7 +8007,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Дописать запросы в семантику страницы (title/H1/текст), отдельную не создавать</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8040,7 +8040,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Дописать запросы в семантику страницы (title/H1/текст), отдельную не создавать</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8073,7 +8073,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8106,7 +8106,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Дописать запросы в семантику страницы (title/H1/текст), отдельную не создавать</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8172,7 +8172,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Дописать запросы в семантику страницы (title/H1/текст), отдельную не создавать</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8205,7 +8205,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Дописать запросы в семантику страницы (title/H1/текст), отдельную не создавать</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8238,7 +8238,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Дописать запросы в семантику страницы (title/H1/текст), отдельную не создавать</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8271,7 +8271,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Дописать запросы в семантику страницы (title/H1/текст), отдельную не создавать</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8304,7 +8304,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Дописать запросы в семантику страницы (title/H1/текст), отдельную не создавать</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8337,7 +8337,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Дописать запросы в семантику страницы (title/H1/текст), отдельную не создавать</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8370,7 +8370,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8403,7 +8403,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8436,7 +8436,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8469,7 +8469,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8535,7 +8535,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Дописать запросы в семантику страницы (title/H1/текст), отдельную не создавать</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8568,7 +8568,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Дописать запросы в семантику страницы (title/H1/текст), отдельную не создавать</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8634,7 +8634,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8667,7 +8667,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8700,7 +8700,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Дописать запросы в семантику страницы (title/H1/текст), отдельную не создавать</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8733,7 +8733,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8766,7 +8766,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Дописать запросы в семантику страницы (title/H1/текст), отдельную не создавать</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8865,7 +8865,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Дописать запросы в семантику страницы (title/H1/текст), отдельную не создавать</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>
@@ -8898,7 +8898,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Оптимизировать (title, H1, текст, фильтры) под кластер</t>
+          <t>Оптимизировать страницу (title, H1, текст) под запросы кластеров</t>
         </is>
       </c>
     </row>

</xml_diff>